<commit_message>
Add Thai BIM 0.20 concrete member sheets and actual reinforcement drawings
</commit_message>
<xml_diff>
--- a/examples/extensions/thai_bim/examples/stair-Circular-BBS.xlsx
+++ b/examples/extensions/thai_bim/examples/stair-Circular-BBS.xlsx
@@ -228,7 +228,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -440,7 +440,7 @@
       </c>
       <c r="N4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O4" s="0" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="N6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O6" s="0" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="N7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O7" s="0" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O8" s="0" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="N9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O9" s="0" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O10" s="0" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="N11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O11" s="0" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="N12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O12" s="0" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="N13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O13" s="0" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="N14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="O14" s="0" t="inlineStr">
@@ -1646,12 +1646,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">467871d9d1254b79</t>
+          <t xml:space="preserve">5764242274554d45</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -1719,12 +1719,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9511c5ea510941d9</t>
+          <t xml:space="preserve">a4e4c7994fbe4c4f</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -1792,12 +1792,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">11cd628075964f77</t>
+          <t xml:space="preserve">b07515b4fd494314</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -1865,12 +1865,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fc575940b19d4bf0</t>
+          <t xml:space="preserve">4dd219bbd6bc46d6</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -1938,12 +1938,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c6ff1ee26dfc45e1</t>
+          <t xml:space="preserve">695f23a7640e41b2</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -2011,12 +2011,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a0239412fc8e4a65</t>
+          <t xml:space="preserve">a726f49fa10d487e</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -2084,12 +2084,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5622351a1a8e4d9f</t>
+          <t xml:space="preserve">7775793f413e4764</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -2157,12 +2157,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d87d6f344358479f</t>
+          <t xml:space="preserve">f2a47b4358eb4327</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -2230,12 +2230,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">edc5c7a30c97496d</t>
+          <t xml:space="preserve">26653aee2b08401a</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -2303,12 +2303,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1918b6e7c3764638</t>
+          <t xml:space="preserve">78d74784490b40e1</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -2376,12 +2376,12 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3257c5fcc27245fe</t>
+          <t xml:space="preserve">78d9dc92f496473b</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">57a1fbeb0ac54b00</t>
+          <t xml:space="preserve">7e0457e882f846f8</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -2522,12 +2522,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eab492ba99294c0d</t>
+          <t xml:space="preserve">d19a1eea3e464cfb</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -2595,12 +2595,12 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f422601ddf954522</t>
+          <t xml:space="preserve">0d2dec145def4d73</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -2668,12 +2668,12 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a6db5b6d8f324843</t>
+          <t xml:space="preserve">2305ef65f78145e4</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -2741,12 +2741,12 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ba6a0c784da24e48</t>
+          <t xml:space="preserve">b96a2784fc2741db</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -2814,12 +2814,12 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6511678a99084313</t>
+          <t xml:space="preserve">8983cb4acd8e49cf</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -2887,12 +2887,12 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e1dc1682e25421c</t>
+          <t xml:space="preserve">511a9195c3264026</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -2960,12 +2960,12 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">88af3c3eafc34258</t>
+          <t xml:space="preserve">853ad7160deb4aa7</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -3033,12 +3033,12 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2e44cccd247f4fce</t>
+          <t xml:space="preserve">734cf69f7756478a</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -3106,12 +3106,12 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0cc7bdf8723241a4</t>
+          <t xml:space="preserve">1429dc156cf44aa5</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -3179,12 +3179,12 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">beb7cc7fe6724b70</t>
+          <t xml:space="preserve">86ffaf8a711d47ba</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -3252,12 +3252,12 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">58c03eef4baa464e</t>
+          <t xml:space="preserve">77992d0a35594dfb</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -3325,12 +3325,12 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cdb1977c52e14908</t>
+          <t xml:space="preserve">9c18097072c24f83</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -3398,12 +3398,12 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">36b410dbc893406d</t>
+          <t xml:space="preserve">8a71fe3cd0bd49c2</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -3471,12 +3471,12 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">14a79335581f4763</t>
+          <t xml:space="preserve">02ff99e31657441f</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -3544,12 +3544,12 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">82b543b7bc2746c1</t>
+          <t xml:space="preserve">7f4ede89d94f4bb6</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -3617,12 +3617,12 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">dcd84662ccf9497e</t>
+          <t xml:space="preserve">8e862951d8e842a6</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -3690,12 +3690,12 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97b6b3b8b50c4211</t>
+          <t xml:space="preserve">304050ba9a834bd6</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -3763,12 +3763,12 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ced7ad821b714b73</t>
+          <t xml:space="preserve">fcbbb35ed08c4817</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -3836,12 +3836,12 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">991c17b645894418</t>
+          <t xml:space="preserve">bad1487ea52b46c4</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -3909,12 +3909,12 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">caecf4198cee41fb</t>
+          <t xml:space="preserve">dda1cf302d4d428f</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -3982,12 +3982,12 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a60a1d82754241e3</t>
+          <t xml:space="preserve">1751f622065948a6</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -4055,12 +4055,12 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3c17fb8ceef74fa5</t>
+          <t xml:space="preserve">2bf271daac064eba</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -4128,12 +4128,12 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3df7061f394441d1</t>
+          <t xml:space="preserve">efdea51c208c434d</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -4201,12 +4201,12 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9641d19471d64371</t>
+          <t xml:space="preserve">62a89aa0dad54f7b</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -4274,12 +4274,12 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac07713cf70f40d2</t>
+          <t xml:space="preserve">4147cbba5189493f</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -4347,12 +4347,12 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">544deac9ac50486a</t>
+          <t xml:space="preserve">c025a2b7dd9d4f46</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -4420,12 +4420,12 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ccd8bfb63a864cf2</t>
+          <t xml:space="preserve">d164ed21c4484742</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -4493,12 +4493,12 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f58291190dec47d3</t>
+          <t xml:space="preserve">c99865566ba94c7e</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -4566,12 +4566,12 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7218e38faf3046a7</t>
+          <t xml:space="preserve">bbf721cf9e154dec</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -4639,12 +4639,12 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">796eca0d7d4e4935</t>
+          <t xml:space="preserve">bd3fbec1a3ff4216</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -4712,12 +4712,12 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ab881847194a4995</t>
+          <t xml:space="preserve">81a18780ef9e4b91</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -4785,12 +4785,12 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f7995437e5284fdb</t>
+          <t xml:space="preserve">cf8c352990a1433d</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -4858,12 +4858,12 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3dc49dfe1304431c</t>
+          <t xml:space="preserve">f1e87b71faf84f85</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -4931,12 +4931,12 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0c9e1e7944cf4e5c</t>
+          <t xml:space="preserve">e01b8c85633a428f</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -5004,12 +5004,12 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8814d4bef6834486</t>
+          <t xml:space="preserve">cea3449b988c4ac0</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -5077,12 +5077,12 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">109220981d1945d1</t>
+          <t xml:space="preserve">24cd7856f21f4601</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -5150,12 +5150,12 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9610e054710f448e</t>
+          <t xml:space="preserve">cfc305c0b0534b62</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -5223,12 +5223,12 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c4f51988a7244536</t>
+          <t xml:space="preserve">23cc4bd387b44a00</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -5296,12 +5296,12 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">93cee391722948dd</t>
+          <t xml:space="preserve">4a03f0773a3847db</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -5369,12 +5369,12 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a9995715af34d8a</t>
+          <t xml:space="preserve">8047c94843474fdb</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -5442,12 +5442,12 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a4ea2767e21247c1</t>
+          <t xml:space="preserve">91e831ae2d104a3b</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -5515,12 +5515,12 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">88bdb67347284256</t>
+          <t xml:space="preserve">449ecf117abf4aa1</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -5588,12 +5588,12 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0d1bd29ba5ae494a</t>
+          <t xml:space="preserve">d9bab95f620340d5</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -5661,12 +5661,12 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">67ec739c8c37484a</t>
+          <t xml:space="preserve">bbe012dff460478c</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -5734,12 +5734,12 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c8cd64e994834616</t>
+          <t xml:space="preserve">f7fa11e6de36420f</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -5807,12 +5807,12 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a1a3b5e0c9a4752</t>
+          <t xml:space="preserve">5ab7a5cf60b641ea</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -5880,12 +5880,12 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">279259ad81b24d26</t>
+          <t xml:space="preserve">c43f197942c14b44</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -5953,12 +5953,12 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">da25f71b43e74083</t>
+          <t xml:space="preserve">6b3890a24a7140e5</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -6026,12 +6026,12 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">918a95d8a2a34486</t>
+          <t xml:space="preserve">67c935827066475f</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -6099,12 +6099,12 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b8dacf0fff2e4f28</t>
+          <t xml:space="preserve">557e8929ba0e4275</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -6172,12 +6172,12 @@
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">24b3739278d64b0e</t>
+          <t xml:space="preserve">fdad535e591d4c96</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -6245,12 +6245,12 @@
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">55b2a2520cec4a47</t>
+          <t xml:space="preserve">e0af190c46984746</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -6318,12 +6318,12 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4faef9ab24fa406a</t>
+          <t xml:space="preserve">8d230b0c8f314091</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -6391,12 +6391,12 @@
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c37c5f2894e74e0b</t>
+          <t xml:space="preserve">95a0c19f312043de</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -6464,12 +6464,12 @@
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">649c2e8caa7d49f6</t>
+          <t xml:space="preserve">a01bb7c6fdd24a56</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -6537,12 +6537,12 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ff52e422a9eb4e0c</t>
+          <t xml:space="preserve">52a2e09c1ead4658</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -6610,12 +6610,12 @@
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1a5105113d664088</t>
+          <t xml:space="preserve">f9985b9e12904bb5</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -6683,12 +6683,12 @@
     <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d4cdec51f6554d18</t>
+          <t xml:space="preserve">b6f91234e9094b43</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -6756,12 +6756,12 @@
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bd5031fcc07f4638</t>
+          <t xml:space="preserve">e7391b59e3764440</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -6829,12 +6829,12 @@
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5d3b55a283ee43fc</t>
+          <t xml:space="preserve">a3aa0e455c6c4b07</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -6902,12 +6902,12 @@
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">33c0e82d43514cc1</t>
+          <t xml:space="preserve">d010e8249cb1427f</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -6975,12 +6975,12 @@
     <row r="75">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e6c4a01aceff48b0</t>
+          <t xml:space="preserve">63b4c59c3549448a</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -7048,12 +7048,12 @@
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ebb0bfbcce8e460a</t>
+          <t xml:space="preserve">87a49b766487498a</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -7121,12 +7121,12 @@
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">67080d073e454f37</t>
+          <t xml:space="preserve">395c8e6cd01c4a7c</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -7194,12 +7194,12 @@
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c1e1ffe594e24495</t>
+          <t xml:space="preserve">99d3294afec04cc1</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -7267,12 +7267,12 @@
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f535003424c74e94</t>
+          <t xml:space="preserve">b46eddbf6a3c4665</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f31ae0157b9b4f0a</t>
+          <t xml:space="preserve">7a770e97fa084f54</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">

</xml_diff>